<commit_message>
Admin: edit data/shala-admissions.xlsx via table editor
</commit_message>
<xml_diff>
--- a/data/shala-admissions.xlsx
+++ b/data/shala-admissions.xlsx
@@ -427,13 +427,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="C2" t="str">
-        <v>Admissions Open Now</v>
+        <v>Teachers Enrollment is OPEN</v>
       </c>
       <c r="D2" t="str">
-        <v>Enroll your child in Sankalp Marathi Shala for the upcoming academic year (September – June). Open to children aged 4 and above.</v>
+        <v>Teacher enrollment is officially open for the upcoming term! Secure your spot today to access new resources, professional development, and community support.</v>
       </c>
       <c r="E2" t="str">
         <v>Email Us to Enroll</v>

</xml_diff>